<commit_message>
Add SOH report for 2026-10-24
</commit_message>
<xml_diff>
--- a/reports/SOH_24_10_2026.xlsx
+++ b/reports/SOH_24_10_2026.xlsx
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>8856</v>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>8856</v>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>8855.5</v>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>8855.5</v>
@@ -10418,7 +10418,7 @@
         </is>
       </c>
       <c r="D360" s="2" t="n">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="E360" s="3" t="n">
         <v>8597</v>

</xml_diff>